<commit_message>
Add pattern matching to program exclusions, add EHA exclusion
program_exclusions.xlsx now supports a Match Type column:
- "exact" (default) — Program Name must match exactly
- "contains" — matches any program containing the value (case-insensitive)

Added EHA as a "contains" exclusion so all programs with EHA in the
name (e.g., Charlotte-VA Supportive Services-SSVF-EHA) automatically
get SOAR/ShallowSub/HUDVASH/Recert fields blanked out.

https://claude.ai/code/session_01JA9wAKoEn1hihmhgHjy4Ab
</commit_message>
<xml_diff>
--- a/config/program_exclusions.xlsx
+++ b/config/program_exclusions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,6 +429,11 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Match Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -446,6 +451,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>VA Suicide Prevention — no SOAR/ShallowSub/HUDVASH/Recert</t>
         </is>
       </c>
@@ -463,6 +473,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>SHIP program</t>
         </is>
       </c>
@@ -480,7 +495,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>CDBG program</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EHA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>non_ssvf</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>All EHA programs — matches any program with EHA in the name</t>
         </is>
       </c>
     </row>

</xml_diff>